<commit_message>
10.0 Tests and translations
</commit_message>
<xml_diff>
--- a/Repository/Settings/RepositoryTranslations.xlsx
+++ b/Repository/Settings/RepositoryTranslations.xlsx
@@ -16,7 +16,7 @@
     <sheet name="RepositoryTranslations" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">RepositoryTranslations!$A$1:$E$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">RepositoryTranslations!$A$1:$E$223</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -1726,7 +1726,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E149"/>
+  <dimension ref="A1:E223"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -3824,12 +3824,1640 @@
         <v>217</v>
       </c>
     </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AIAssistantName</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Report Designer</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Concepteur de rapports</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AIAssistantName</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule &amp; Output</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planification et sortie</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AIAssistantName</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data Analyst</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Analyste de données</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AIAssistantName</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">System Admin</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Administrateur système</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">List all available data sources and their tables</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lister toutes les sources de données disponibles et leurs tables</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What columns are in the [table] table?</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quelles colonnes contient la table [table] ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show me a sample of data from [table]</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Montre-moi un échantillon de données de [table]</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How many rows are in [table]?</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Combien de lignes y a-t-il dans [table] ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">List all reports available</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lister tous les rapports disponibles</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Can you write an executive summary of 200 words based on data got from Overview Sales report</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peux-tu rédiger une synthèse de 200 mots à partir des données du rapport Overview Sales ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For Northwind, create a report showing total sales by category</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour Northwind, crée un rapport affichant les ventes totales par catégorie</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For Northwind, build a monthly sales trend report for this year</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour Northwind, construis un rapport de tendance mensuelle des ventes pour cette année</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For Northwind, create a top 10 customers report ranked by revenue</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour Northwind, crée un rapport des 10 meilleurs clients classés par chiffre d'affaires</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For Northwind, create a sales report filtered by date range</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour Northwind, crée un rapport des ventes filtré par plage de dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Save the report created in the Sales folder</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enregistre le rapport créé dans le dossier Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Create a report with the SQL and save it in the Marketing folder</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crée un rapport avec le SQL et enregistre-le dans le dossier Marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Save the report in Reports\Monthly Summary.srex</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enregistre le rapport dans Reports\Monthly Summary.srex</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Create a default Excel output for the [report name] report and save the result in my Personal Folder</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crée une sortie Excel par défaut pour le rapport [report name] et enregistre le résultat dans mon dossier personnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule the output of [report name] every Monday at 9am</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planifie la sortie de [report name] tous les lundis à 9h</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For Northwind, make a report with a bar chart of orders by country</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour Northwind, crée un rapport avec un graphique à barres des commandes par pays</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For Northwind, add a line chart showing the sales trend over time</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour Northwind, ajoute un graphique en courbes montrant la tendance des ventes dans le temps</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For Northwind, show the revenue breakdown by category as a pie chart</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour Northwind, affiche la répartition du chiffre d'affaires par catégorie sous forme de camembert</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For Northwind, add a bar chart comparing sales across regions</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour Northwind, ajoute un graphique à barres comparant les ventes entre régions</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For Northwind, write a query to show total sales per month</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour Northwind, écris une requête affichant les ventes totales par mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For Northwind, write a query to find the top 10 products by revenue</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour Northwind, écris une requête pour trouver les 10 meilleurs produits par chiffre d'affaires</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For Northwind, write a query to show orders placed in the last 30 days</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour Northwind, écris une requête affichant les commandes passées au cours des 30 derniers jours</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What were total sales last month?</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quelles ont été les ventes totales le mois dernier ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show me the top 10 customers by revenue</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Montre-moi les 10 meilleurs clients par chiffre d'affaires</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Which products are selling the most this year?</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quels produits se vendent le mieux cette année ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What is the sales trend over the last 6 months?</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quelle est la tendance des ventes sur les 6 derniers mois ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compare sales across regions for this quarter</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compare les ventes entre régions pour ce trimestre</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Give me an executive summary of the sales overview report</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Donne-moi une synthèse du rapport de synthèse des ventes</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Summarize the key findings from the [report name] report</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Résume les principales conclusions du rapport [report name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What are the main trends in the [report name] data?</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quelles sont les principales tendances dans les données de [report name] ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Which category has the highest growth compared to last year?</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quelle catégorie a la plus forte croissance par rapport à l'année dernière ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are there any anomalies in the latest [report name] results?</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y a-t-il des anomalies dans les derniers résultats de [report name] ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What does the data say about [business question]?</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Que disent les données à propos de [business question] ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show me today's event log</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Montre-moi le journal des événements d'aujourd'hui</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show errors in today's event log</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Affiche les erreurs dans le journal des événements d'aujourd'hui</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show failed authentication attempts today</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Affiche les tentatives d'authentification échouées aujourd'hui</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show executions log for [date]</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Affiche le journal des exécutions pour [date]</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Search the executions log for [report name]</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recherche [report name] dans le journal des exécutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show today's schedule log</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Affiche le journal des planifications d'aujourd'hui</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show me all users and their groups</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Montre-moi tous les utilisateurs et leurs groupes</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Who belongs to the [group name] group?</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qui appartient au groupe [group name] ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show the configuration summary</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Affiche le résumé de la configuration</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run the Audit report</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exécute le rapport Audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run the Security report</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exécute le rapport Security</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run the Activity report</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exécute le rapport Activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show me recent report executions from the Activity report</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Montre-moi les exécutions de rapports récentes à partir du rapport Activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Are there any errors in today's logs?</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y a-t-il des erreurs dans les journaux d'aujourd'hui ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show me all authentication failures this week</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Montre-moi tous les échecs d'authentification de cette semaine</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Which reports failed to execute today?</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quels rapports ont échoué à s'exécuter aujourd'hui ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For [source], create a report showing total sales by category</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour [source], crée un rapport affichant les ventes totales par catégorie</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For [source], build a monthly sales trend report for this year</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour [source], construis un rapport de tendance mensuelle des ventes pour cette année</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For [source], create a top 10 customers report ranked by revenue</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour [source], crée un rapport des 10 meilleurs clients classés par chiffre d'affaires</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For [source], make a report with a bar chart of orders by country</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour [source], crée un rapport avec un graphique à barres des commandes par pays</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For [source], create a report with a pie chart of revenue by region</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pour [source], crée un rapport avec un camembert du chiffre d'affaires par région</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add a date restriction to the [report name] report</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ajoute une restriction de date au rapport [report name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add a bar chart to the [report name] report</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ajoute un graphique à barres au rapport [report name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rename the [report name] report to [new name]</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Renomme le rapport [report name] en [new name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Move the [report name] report to the [folder] folder</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Déplace le rapport [report name] vers le dossier [folder]</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Create an Excel output for [report name] saved in my Personal folder</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crée une sortie Excel pour [report name] enregistrée dans mon dossier personnel</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Create a PDF output for [report name] saved in C:\Reports\Daily</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crée une sortie PDF pour [report name] enregistrée dans C:\Reports\Daily</t>
+        </is>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Change the output format of [report name] to CSV</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Change le format de sortie de [report name] en CSV</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Remove the output from [report name]</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supprime la sortie de [report name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule [report name] to run every Monday at 8am</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planifie [report name] pour s'exécuter tous les lundis à 8h</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule [report name] to run every day at 7am</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planifie [report name] pour s'exécuter tous les jours à 7h</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule [report name] every Monday at 9am</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planifie [report name] tous les lundis à 9h</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule [report name] on the 1st of every month at 6am</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planifie [report name] le 1er de chaque mois à 6h</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run [report name] once tomorrow at 3pm</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exécute [report name] une fois demain à 15h</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Delete the schedule for [report name]</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Supprime la planification de [report name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show me the outputs and schedules configured for [report name]</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Montre-moi les sorties et planifications configurées pour [report name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">*</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">List all reports that have a schedule</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lister tous les rapports qui ont une planification</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E149" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E149">
-      <sortCondition ref="A2:A149"/>
-      <sortCondition ref="B2:B149"/>
-      <sortCondition ref="C2:C149"/>
+  <autoFilter ref="A1:E223" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E223">
+      <sortCondition ref="A2:A223"/>
+      <sortCondition ref="B2:B223"/>
+      <sortCondition ref="C2:C223"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
10.0 rename Assistant to Agent
</commit_message>
<xml_diff>
--- a/Repository/Settings/RepositoryTranslations.xlsx
+++ b/Repository/Settings/RepositoryTranslations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_dev\Seal-Report\Repository\Settings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBDAFC75-CF72-4745-BB1B-9562A59786F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FD962C2-30AB-40B5-A4B0-5FBF65A74892}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18270" yWindow="2220" windowWidth="24375" windowHeight="15855" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -874,9 +874,6 @@
     <t>Les lundis à 6:00</t>
   </si>
   <si>
-    <t>AIAssistantName</t>
-  </si>
-  <si>
     <t>Report Designer</t>
   </si>
   <si>
@@ -1324,9 +1321,6 @@
     <t>Lister tous les rapports qui ont une planification</t>
   </si>
   <si>
-    <t>AIAssistantDescription</t>
-  </si>
-  <si>
     <t>Designs and builds reports from natural-language requests: explores data sources, validates SQL, and creates SQL-based or metadata-based reports.</t>
   </si>
   <si>
@@ -1349,6 +1343,12 @@
   </si>
   <si>
     <t>Gère l'administration et le dépannage : lit les journaux d'événements, d'exécution et de planification, inspecte les rapports et les sources, et gère les fichiers du référentiel.</t>
+  </si>
+  <si>
+    <t>AIAgentDescription</t>
+  </si>
+  <si>
+    <t>AIAgentName</t>
   </si>
 </sst>
 </file>
@@ -4303,1094 +4303,1094 @@
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
+        <v>441</v>
+      </c>
+      <c r="B150" t="s">
+        <v>266</v>
+      </c>
+      <c r="C150" t="s">
         <v>283</v>
       </c>
-      <c r="B150" t="s">
-        <v>266</v>
-      </c>
-      <c r="C150" t="s">
+      <c r="E150" t="s">
         <v>284</v>
-      </c>
-      <c r="E150" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>283</v>
+        <v>441</v>
       </c>
       <c r="B151" t="s">
         <v>266</v>
       </c>
       <c r="C151" t="s">
+        <v>285</v>
+      </c>
+      <c r="E151" t="s">
         <v>286</v>
-      </c>
-      <c r="E151" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>283</v>
+        <v>441</v>
       </c>
       <c r="B152" t="s">
         <v>266</v>
       </c>
       <c r="C152" t="s">
+        <v>287</v>
+      </c>
+      <c r="E152" t="s">
         <v>288</v>
-      </c>
-      <c r="E152" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>283</v>
+        <v>441</v>
       </c>
       <c r="B153" t="s">
         <v>266</v>
       </c>
       <c r="C153" t="s">
+        <v>289</v>
+      </c>
+      <c r="E153" t="s">
         <v>290</v>
-      </c>
-      <c r="E153" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
+        <v>291</v>
+      </c>
+      <c r="B154" t="s">
+        <v>266</v>
+      </c>
+      <c r="C154" t="s">
         <v>292</v>
       </c>
-      <c r="B154" t="s">
-        <v>266</v>
-      </c>
-      <c r="C154" t="s">
+      <c r="E154" t="s">
         <v>293</v>
-      </c>
-      <c r="E154" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B155" t="s">
         <v>266</v>
       </c>
       <c r="C155" t="s">
+        <v>294</v>
+      </c>
+      <c r="E155" t="s">
         <v>295</v>
-      </c>
-      <c r="E155" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B156" t="s">
         <v>266</v>
       </c>
       <c r="C156" t="s">
+        <v>296</v>
+      </c>
+      <c r="E156" t="s">
         <v>297</v>
-      </c>
-      <c r="E156" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B157" t="s">
         <v>266</v>
       </c>
       <c r="C157" t="s">
+        <v>298</v>
+      </c>
+      <c r="E157" t="s">
         <v>299</v>
-      </c>
-      <c r="E157" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B158" t="s">
         <v>266</v>
       </c>
       <c r="C158" t="s">
+        <v>300</v>
+      </c>
+      <c r="E158" t="s">
         <v>301</v>
-      </c>
-      <c r="E158" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B159" t="s">
         <v>266</v>
       </c>
       <c r="C159" t="s">
+        <v>302</v>
+      </c>
+      <c r="E159" t="s">
         <v>303</v>
-      </c>
-      <c r="E159" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B160" t="s">
         <v>266</v>
       </c>
       <c r="C160" t="s">
+        <v>304</v>
+      </c>
+      <c r="E160" t="s">
         <v>305</v>
-      </c>
-      <c r="E160" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B161" t="s">
         <v>266</v>
       </c>
       <c r="C161" t="s">
+        <v>306</v>
+      </c>
+      <c r="E161" t="s">
         <v>307</v>
-      </c>
-      <c r="E161" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B162" t="s">
         <v>266</v>
       </c>
       <c r="C162" t="s">
+        <v>308</v>
+      </c>
+      <c r="E162" t="s">
         <v>309</v>
-      </c>
-      <c r="E162" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B163" t="s">
         <v>266</v>
       </c>
       <c r="C163" t="s">
+        <v>310</v>
+      </c>
+      <c r="E163" t="s">
         <v>311</v>
-      </c>
-      <c r="E163" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B164" t="s">
         <v>266</v>
       </c>
       <c r="C164" t="s">
+        <v>312</v>
+      </c>
+      <c r="E164" t="s">
         <v>313</v>
-      </c>
-      <c r="E164" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B165" t="s">
         <v>266</v>
       </c>
       <c r="C165" t="s">
+        <v>314</v>
+      </c>
+      <c r="E165" t="s">
         <v>315</v>
-      </c>
-      <c r="E165" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B166" t="s">
         <v>266</v>
       </c>
       <c r="C166" t="s">
+        <v>316</v>
+      </c>
+      <c r="E166" t="s">
         <v>317</v>
-      </c>
-      <c r="E166" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B167" t="s">
         <v>266</v>
       </c>
       <c r="C167" t="s">
+        <v>318</v>
+      </c>
+      <c r="E167" t="s">
         <v>319</v>
-      </c>
-      <c r="E167" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B168" t="s">
         <v>266</v>
       </c>
       <c r="C168" t="s">
+        <v>320</v>
+      </c>
+      <c r="E168" t="s">
         <v>321</v>
-      </c>
-      <c r="E168" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B169" t="s">
         <v>266</v>
       </c>
       <c r="C169" t="s">
+        <v>322</v>
+      </c>
+      <c r="E169" t="s">
         <v>323</v>
-      </c>
-      <c r="E169" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B170" t="s">
         <v>266</v>
       </c>
       <c r="C170" t="s">
+        <v>324</v>
+      </c>
+      <c r="E170" t="s">
         <v>325</v>
-      </c>
-      <c r="E170" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B171" t="s">
         <v>266</v>
       </c>
       <c r="C171" t="s">
+        <v>326</v>
+      </c>
+      <c r="E171" t="s">
         <v>327</v>
-      </c>
-      <c r="E171" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B172" t="s">
         <v>266</v>
       </c>
       <c r="C172" t="s">
+        <v>328</v>
+      </c>
+      <c r="E172" t="s">
         <v>329</v>
-      </c>
-      <c r="E172" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B173" t="s">
         <v>266</v>
       </c>
       <c r="C173" t="s">
+        <v>330</v>
+      </c>
+      <c r="E173" t="s">
         <v>331</v>
-      </c>
-      <c r="E173" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B174" t="s">
         <v>266</v>
       </c>
       <c r="C174" t="s">
+        <v>332</v>
+      </c>
+      <c r="E174" t="s">
         <v>333</v>
-      </c>
-      <c r="E174" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B175" t="s">
         <v>266</v>
       </c>
       <c r="C175" t="s">
+        <v>334</v>
+      </c>
+      <c r="E175" t="s">
         <v>335</v>
-      </c>
-      <c r="E175" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B176" t="s">
         <v>266</v>
       </c>
       <c r="C176" t="s">
+        <v>336</v>
+      </c>
+      <c r="E176" t="s">
         <v>337</v>
-      </c>
-      <c r="E176" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B177" t="s">
         <v>266</v>
       </c>
       <c r="C177" t="s">
+        <v>338</v>
+      </c>
+      <c r="E177" t="s">
         <v>339</v>
-      </c>
-      <c r="E177" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B178" t="s">
         <v>266</v>
       </c>
       <c r="C178" t="s">
+        <v>340</v>
+      </c>
+      <c r="E178" t="s">
         <v>341</v>
-      </c>
-      <c r="E178" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B179" t="s">
         <v>266</v>
       </c>
       <c r="C179" t="s">
+        <v>342</v>
+      </c>
+      <c r="E179" t="s">
         <v>343</v>
-      </c>
-      <c r="E179" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B180" t="s">
         <v>266</v>
       </c>
       <c r="C180" t="s">
+        <v>344</v>
+      </c>
+      <c r="E180" t="s">
         <v>345</v>
-      </c>
-      <c r="E180" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B181" t="s">
         <v>266</v>
       </c>
       <c r="C181" t="s">
+        <v>346</v>
+      </c>
+      <c r="E181" t="s">
         <v>347</v>
-      </c>
-      <c r="E181" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B182" t="s">
         <v>266</v>
       </c>
       <c r="C182" t="s">
+        <v>348</v>
+      </c>
+      <c r="E182" t="s">
         <v>349</v>
-      </c>
-      <c r="E182" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B183" t="s">
         <v>266</v>
       </c>
       <c r="C183" t="s">
+        <v>350</v>
+      </c>
+      <c r="E183" t="s">
         <v>351</v>
-      </c>
-      <c r="E183" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B184" t="s">
         <v>266</v>
       </c>
       <c r="C184" t="s">
+        <v>352</v>
+      </c>
+      <c r="E184" t="s">
         <v>353</v>
-      </c>
-      <c r="E184" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B185" t="s">
         <v>266</v>
       </c>
       <c r="C185" t="s">
+        <v>354</v>
+      </c>
+      <c r="E185" t="s">
         <v>355</v>
-      </c>
-      <c r="E185" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B186" t="s">
         <v>266</v>
       </c>
       <c r="C186" t="s">
+        <v>356</v>
+      </c>
+      <c r="E186" t="s">
         <v>357</v>
-      </c>
-      <c r="E186" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B187" t="s">
         <v>266</v>
       </c>
       <c r="C187" t="s">
+        <v>358</v>
+      </c>
+      <c r="E187" t="s">
         <v>359</v>
-      </c>
-      <c r="E187" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B188" t="s">
         <v>266</v>
       </c>
       <c r="C188" t="s">
+        <v>360</v>
+      </c>
+      <c r="E188" t="s">
         <v>361</v>
-      </c>
-      <c r="E188" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B189" t="s">
         <v>266</v>
       </c>
       <c r="C189" t="s">
+        <v>362</v>
+      </c>
+      <c r="E189" t="s">
         <v>363</v>
-      </c>
-      <c r="E189" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B190" t="s">
         <v>266</v>
       </c>
       <c r="C190" t="s">
+        <v>364</v>
+      </c>
+      <c r="E190" t="s">
         <v>365</v>
-      </c>
-      <c r="E190" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B191" t="s">
         <v>266</v>
       </c>
       <c r="C191" t="s">
+        <v>366</v>
+      </c>
+      <c r="E191" t="s">
         <v>367</v>
-      </c>
-      <c r="E191" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B192" t="s">
         <v>266</v>
       </c>
       <c r="C192" t="s">
+        <v>368</v>
+      </c>
+      <c r="E192" t="s">
         <v>369</v>
-      </c>
-      <c r="E192" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B193" t="s">
         <v>266</v>
       </c>
       <c r="C193" t="s">
+        <v>370</v>
+      </c>
+      <c r="E193" t="s">
         <v>371</v>
-      </c>
-      <c r="E193" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B194" t="s">
         <v>266</v>
       </c>
       <c r="C194" t="s">
+        <v>372</v>
+      </c>
+      <c r="E194" t="s">
         <v>373</v>
-      </c>
-      <c r="E194" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B195" t="s">
         <v>266</v>
       </c>
       <c r="C195" t="s">
+        <v>374</v>
+      </c>
+      <c r="E195" t="s">
         <v>375</v>
-      </c>
-      <c r="E195" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B196" t="s">
         <v>266</v>
       </c>
       <c r="C196" t="s">
+        <v>376</v>
+      </c>
+      <c r="E196" t="s">
         <v>377</v>
-      </c>
-      <c r="E196" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B197" t="s">
         <v>266</v>
       </c>
       <c r="C197" t="s">
+        <v>378</v>
+      </c>
+      <c r="E197" t="s">
         <v>379</v>
-      </c>
-      <c r="E197" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B198" t="s">
         <v>266</v>
       </c>
       <c r="C198" t="s">
+        <v>380</v>
+      </c>
+      <c r="E198" t="s">
         <v>381</v>
-      </c>
-      <c r="E198" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B199" t="s">
         <v>266</v>
       </c>
       <c r="C199" t="s">
+        <v>382</v>
+      </c>
+      <c r="E199" t="s">
         <v>383</v>
-      </c>
-      <c r="E199" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B200" t="s">
         <v>266</v>
       </c>
       <c r="C200" t="s">
+        <v>384</v>
+      </c>
+      <c r="E200" t="s">
         <v>385</v>
-      </c>
-      <c r="E200" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B201" t="s">
         <v>266</v>
       </c>
       <c r="C201" t="s">
+        <v>386</v>
+      </c>
+      <c r="E201" t="s">
         <v>387</v>
-      </c>
-      <c r="E201" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B202" t="s">
         <v>266</v>
       </c>
       <c r="C202" t="s">
+        <v>388</v>
+      </c>
+      <c r="E202" t="s">
         <v>389</v>
-      </c>
-      <c r="E202" t="s">
-        <v>390</v>
       </c>
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B203" t="s">
         <v>266</v>
       </c>
       <c r="C203" t="s">
+        <v>390</v>
+      </c>
+      <c r="E203" t="s">
         <v>391</v>
-      </c>
-      <c r="E203" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B204" t="s">
         <v>266</v>
       </c>
       <c r="C204" t="s">
+        <v>392</v>
+      </c>
+      <c r="E204" t="s">
         <v>393</v>
-      </c>
-      <c r="E204" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B205" t="s">
         <v>266</v>
       </c>
       <c r="C205" t="s">
+        <v>394</v>
+      </c>
+      <c r="E205" t="s">
         <v>395</v>
-      </c>
-      <c r="E205" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B206" t="s">
         <v>266</v>
       </c>
       <c r="C206" t="s">
+        <v>396</v>
+      </c>
+      <c r="E206" t="s">
         <v>397</v>
-      </c>
-      <c r="E206" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B207" t="s">
         <v>266</v>
       </c>
       <c r="C207" t="s">
+        <v>398</v>
+      </c>
+      <c r="E207" t="s">
         <v>399</v>
-      </c>
-      <c r="E207" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B208" t="s">
         <v>266</v>
       </c>
       <c r="C208" t="s">
+        <v>400</v>
+      </c>
+      <c r="E208" t="s">
         <v>401</v>
-      </c>
-      <c r="E208" t="s">
-        <v>402</v>
       </c>
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B209" t="s">
         <v>266</v>
       </c>
       <c r="C209" t="s">
+        <v>402</v>
+      </c>
+      <c r="E209" t="s">
         <v>403</v>
-      </c>
-      <c r="E209" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B210" t="s">
         <v>266</v>
       </c>
       <c r="C210" t="s">
+        <v>404</v>
+      </c>
+      <c r="E210" t="s">
         <v>405</v>
-      </c>
-      <c r="E210" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B211" t="s">
         <v>266</v>
       </c>
       <c r="C211" t="s">
+        <v>406</v>
+      </c>
+      <c r="E211" t="s">
         <v>407</v>
-      </c>
-      <c r="E211" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B212" t="s">
         <v>266</v>
       </c>
       <c r="C212" t="s">
+        <v>408</v>
+      </c>
+      <c r="E212" t="s">
         <v>409</v>
-      </c>
-      <c r="E212" t="s">
-        <v>410</v>
       </c>
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B213" t="s">
         <v>266</v>
       </c>
       <c r="C213" t="s">
+        <v>410</v>
+      </c>
+      <c r="E213" t="s">
         <v>411</v>
-      </c>
-      <c r="E213" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B214" t="s">
         <v>266</v>
       </c>
       <c r="C214" t="s">
+        <v>412</v>
+      </c>
+      <c r="E214" t="s">
         <v>413</v>
-      </c>
-      <c r="E214" t="s">
-        <v>414</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B215" t="s">
         <v>266</v>
       </c>
       <c r="C215" t="s">
+        <v>414</v>
+      </c>
+      <c r="E215" t="s">
         <v>415</v>
-      </c>
-      <c r="E215" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B216" t="s">
         <v>266</v>
       </c>
       <c r="C216" t="s">
+        <v>416</v>
+      </c>
+      <c r="E216" t="s">
         <v>417</v>
-      </c>
-      <c r="E216" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B217" t="s">
         <v>266</v>
       </c>
       <c r="C217" t="s">
+        <v>418</v>
+      </c>
+      <c r="E217" t="s">
         <v>419</v>
-      </c>
-      <c r="E217" t="s">
-        <v>420</v>
       </c>
     </row>
     <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B218" t="s">
         <v>266</v>
       </c>
       <c r="C218" t="s">
+        <v>420</v>
+      </c>
+      <c r="E218" t="s">
         <v>421</v>
-      </c>
-      <c r="E218" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B219" t="s">
         <v>266</v>
       </c>
       <c r="C219" t="s">
+        <v>422</v>
+      </c>
+      <c r="E219" t="s">
         <v>423</v>
-      </c>
-      <c r="E219" t="s">
-        <v>424</v>
       </c>
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B220" t="s">
         <v>266</v>
       </c>
       <c r="C220" t="s">
+        <v>424</v>
+      </c>
+      <c r="E220" t="s">
         <v>425</v>
-      </c>
-      <c r="E220" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B221" t="s">
         <v>266</v>
       </c>
       <c r="C221" t="s">
+        <v>426</v>
+      </c>
+      <c r="E221" t="s">
         <v>427</v>
-      </c>
-      <c r="E221" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B222" t="s">
         <v>266</v>
       </c>
       <c r="C222" t="s">
+        <v>428</v>
+      </c>
+      <c r="E222" t="s">
         <v>429</v>
-      </c>
-      <c r="E222" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B223" t="s">
         <v>266</v>
       </c>
       <c r="C223" t="s">
+        <v>430</v>
+      </c>
+      <c r="E223" t="s">
         <v>431</v>
-      </c>
-      <c r="E223" t="s">
-        <v>432</v>
       </c>
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
+        <v>440</v>
+      </c>
+      <c r="B224" t="s">
+        <v>266</v>
+      </c>
+      <c r="C224" t="s">
+        <v>432</v>
+      </c>
+      <c r="E224" t="s">
         <v>433</v>
-      </c>
-      <c r="B224" t="s">
-        <v>266</v>
-      </c>
-      <c r="C224" t="s">
-        <v>434</v>
-      </c>
-      <c r="E224" t="s">
-        <v>435</v>
       </c>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="B225" t="s">
         <v>266</v>
       </c>
       <c r="C225" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="E225" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="B226" t="s">
         <v>266</v>
       </c>
       <c r="C226" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E226" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="B227" t="s">
         <v>266</v>
       </c>
       <c r="C227" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E227" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
10.0 project and js cleanup
</commit_message>
<xml_diff>
--- a/Repository/Settings/RepositoryTranslations.xlsx
+++ b/Repository/Settings/RepositoryTranslations.xlsx
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E229"/>
+  <dimension ref="A1:E260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5984,6 +5984,688 @@
       <c r="E229" t="inlineStr">
         <is>
           <t>Montre-moi les périphériques de sortie que je peux utiliser</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Running a database query</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Exécution d'une requête sur la base de données</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Getting columns of table {table}</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Récupération des colonnes de la table {table}</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Getting sample values of {table}.{column}</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Récupération d'exemples de valeurs de {table}.{column}</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Counting rows of table {table}</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Comptage des lignes de la table {table}</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Listing data sources</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Liste des sources de données</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Inspecting data source {name}</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Analyse de la source de données {name}</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Reading report {path}</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Lecture du rapport {path}</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Reading report definition {path}</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Lecture de la définition du rapport {path}</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Analyzing the report request</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Analyse de la demande de rapport</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Creating report {display_name}</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Création du rapport {display_name}</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Creating report {path}</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Création du rapport {path}</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Listing output devices</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Liste des périphériques de sortie</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Configuring output of report {path}</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Configuration de la sortie du rapport {path}</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Configuring schedule of report {path}</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Configuration de la planification du rapport {path}</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Executing report {path}</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Exécution du rapport {path}</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Browsing files</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Parcours des fichiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Managing file {path}</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Gestion du fichier {path}</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Listing reports</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Liste des rapports</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Getting the current folder</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Récupération du dossier courant</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Reading {type} logs</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Lecture des journaux {type}</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Reading view parameters of {path}</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Lecture des paramètres de vue de {path}</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Configuring view of report {path}</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Configuration de la vue du rapport {path}</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Preparing to build a report from metadata</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Préparation d'un rapport à partir des métadonnées</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Preparing to build a report from SQL</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Préparation d'un rapport à partir du SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Preparing to build a NoSQL report</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Préparation d'un rapport NoSQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Preparing to style the report view</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Préparation de la mise en forme de la vue du rapport</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Preparing to schedule the report delivery</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Préparation de la planification de la diffusion du rapport</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Preparing to analyze the report data</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Préparation de l'analyse des données du rapport</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Preparing to troubleshoot with the logs</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Préparation du diagnostic à partir des journaux</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Preparing to audit security and activity</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Préparation de l'audit de sécurité et d'activité</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>AIToolProgress</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Preparing to manage report files</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Préparation de la gestion des fichiers de rapport</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
10.0 data source agent
</commit_message>
<xml_diff>
--- a/Repository/Settings/RepositoryTranslations.xlsx
+++ b/Repository/Settings/RepositoryTranslations.xlsx
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E260"/>
+  <dimension ref="A1:E271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6666,6 +6666,248 @@
       <c r="E260" t="inlineStr">
         <is>
           <t>Préparation de la gestion des fichiers de rapport</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Which reports use the [column] column?</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Quels rapports utilisent la colonne [column] ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>For [source], add the [table] table</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Pour [source], ajoute la table [table]</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>For [source], add a full name column to the [table] table</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Pour [source], ajoute une colonne nom complet à la table [table]</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>For [source], suggest joins between the tables</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Pour [source], propose des jointures entre les tables</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>For [source], create an enumerated list from the [column] column</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Pour [source], crée une liste de valeurs à partir de la colonne [column]</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>AIAgentName</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Data Source Manager</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Gestionnaire de sources de données</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>AIAgentDescription</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Manages the data source metadata model from natural-language requests: adds tables and columns, builds enumerated lists and joins, edits or removes metadata, and checks which reports are impacted before any change.</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Gère le modèle de métadonnées des sources de données à partir de demandes en langage naturel : ajoute des tables et des colonnes, construit des listes de valeurs et des jointures, modifie ou supprime des métadonnées, et vérifie quels rapports sont impactés avant toute modification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Show the schema of the [source] data source</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Affiche le schéma de la source de données [source]</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>For [source], add a join between [table] and [table]</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Pour [source], ajoute une jointure entre [table] et [table]</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>For [source], change the SQL of the [column] column</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Pour [source], modifie le SQL de la colonne [column]</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>AISamplePrompt</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Remove the [column] column from [source]</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Supprime la colonne [column] de [source]</t>
         </is>
       </c>
     </row>

</xml_diff>